<commit_message>
email send by ui
</commit_message>
<xml_diff>
--- a/emails.xlsx
+++ b/emails.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26626"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27830"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\email_sender_python\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A87939B8-9F27-4D63-8E1B-490D1D1E44F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88438BB8-D68A-4002-B7B4-E3C7FA872189}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>Name</t>
   </si>
@@ -28,22 +28,16 @@
     <t>Email</t>
   </si>
   <si>
-    <t>Test user 1</t>
+    <t>lakshikahirushini89@gmail.com</t>
   </si>
   <si>
-    <t>testUser1@user.com</t>
+    <t>Lakshika</t>
   </si>
   <si>
-    <t>testUser3@user.com</t>
+    <t>Jeewantha</t>
   </si>
   <si>
-    <t>testUser2@user.com</t>
-  </si>
-  <si>
-    <t>Test user 2</t>
-  </si>
-  <si>
-    <t>Test user 3</t>
+    <t>jeewanthamsenanayake@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -320,7 +314,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:B200"/>
+  <dimension ref="A1:B199"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="41.28515625" customWidth="1"/>
@@ -338,27 +332,23 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>3</v>
-      </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>4</v>
-      </c>
+      <c r="A4" s="1"/>
+      <c r="B4" s="1"/>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" s="1"/>
@@ -1140,18 +1130,13 @@
       <c r="A199" s="1"/>
       <c r="B199" s="1"/>
     </row>
-    <row r="200" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A200" s="1"/>
-      <c r="B200" s="1"/>
-    </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1" xr:uid="{A89E8725-FE33-4C9E-B7C2-C63766A869CC}"/>
-    <hyperlink ref="B3" r:id="rId2" xr:uid="{F862EAE9-4F4A-4F87-94BC-D75564D58394}"/>
-    <hyperlink ref="B4" r:id="rId3" xr:uid="{F74D7CB6-5F84-4877-9399-B63E6A6221B7}"/>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{D58CE650-C673-4C3C-8031-92082F60BAAD}"/>
+    <hyperlink ref="B3" r:id="rId2" xr:uid="{0A17E41A-DF81-4F72-B0C1-06DF39DF6202}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId4"/>
+  <pageSetup orientation="portrait" r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
attachment can send by ui
</commit_message>
<xml_diff>
--- a/emails.xlsx
+++ b/emails.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\email_sender_python\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88438BB8-D68A-4002-B7B4-E3C7FA872189}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3112B7A-AB34-4E48-B424-A86404B00D74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,16 +28,16 @@
     <t>Email</t>
   </si>
   <si>
-    <t>lakshikahirushini89@gmail.com</t>
-  </si>
-  <si>
-    <t>Lakshika</t>
-  </si>
-  <si>
     <t>Jeewantha</t>
   </si>
   <si>
     <t>jeewanthamsenanayake@gmail.com</t>
+  </si>
+  <si>
+    <t>en93893@sjp.ac.lk</t>
+  </si>
+  <si>
+    <t>Jeewantha Sjp</t>
   </si>
 </sst>
 </file>
@@ -332,18 +332,18 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A3" s="1" t="s">
-        <v>4</v>
-      </c>
       <c r="B3" s="2" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">

</xml_diff>